<commit_message>
Updated Review matrix sheet
</commit_message>
<xml_diff>
--- a/02_Literature_Review/Literature_Review_Matrix.xlsx
+++ b/02_Literature_Review/Literature_Review_Matrix.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ctutrainingsolutionspt-my.sharepoint.com/personal/lusukama_selemani_ctutraining_co_za/Documents/Documents/POES-LUSUKAMA/Research-2026/Capstone_Project_Pack_with_CTU_Logo/Capstone_Project_Pack/02_Literature_Review/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dylan\Desktop\project github\TrackWIL\02_Literature_Review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{485AF264-7E29-44F8-A03F-95DDEB33E7AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6A24ED2-7C3F-4292-8DBC-6B6BE1EE9C51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="540" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tracker" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="82">
   <si>
     <t>LITERATURE REVIEW MATRIX</t>
   </si>
@@ -56,6 +56,219 @@
   </si>
   <si>
     <t>Reference/URL</t>
+  </si>
+  <si>
+    <t>LR01</t>
+  </si>
+  <si>
+    <t>Schuster, L. and Glavas, C.</t>
+  </si>
+  <si>
+    <t>Exploring the dimensions of electronic work integrated learning (eWIL)</t>
+  </si>
+  <si>
+    <t>Investigates how technology is used to support and deliver Work-Integrated Learning.</t>
+  </si>
+  <si>
+    <t>Systematic literature review of electronic WIL initiatives.</t>
+  </si>
+  <si>
+    <t>Technology can support WIL administration and learning activities. Its role can range from limited administrative support to a central part of the learning experience.</t>
+  </si>
+  <si>
+    <t>The review examines different types of electronic WIL, so its findings do not establish that one particular system is best for every institution.</t>
+  </si>
+  <si>
+    <t>Provides academic background for developing TrackWIL as a digital tool for managing WIL documentation, activities and communication.</t>
+  </si>
+  <si>
+    <t>https://www.sciencedirect.com/science/article/abs/pii/S1747938X17300155</t>
+  </si>
+  <si>
+    <t>LR02</t>
+  </si>
+  <si>
+    <t>InPlace Software</t>
+  </si>
+  <si>
+    <t>n.d.</t>
+  </si>
+  <si>
+    <t>Work Integrated Learning Placement Software</t>
+  </si>
+  <si>
+    <t>Addresses the management, coordination and monitoring of student placements in higher education.</t>
+  </si>
+  <si>
+    <t>Industry software platform for placement management, allocation, compliance, communications and reporting.</t>
+  </si>
+  <si>
+    <t>Provides centralised placement management, placement allocation, student portals, compliance tools and reporting capabilities.</t>
+  </si>
+  <si>
+    <t>Its public product information does not establish whether every TrackWIL-specific daily logbook and mentor verification requirement is available in every deployment.</t>
+  </si>
+  <si>
+    <t>Provides a similar system for comparison and identifies useful features such as centralised records, role-specific access and progress reporting.</t>
+  </si>
+  <si>
+    <t>https://inplacesoftware.com/higher-education/work-integrated-learning/</t>
+  </si>
+  <si>
+    <t>LR03</t>
+  </si>
+  <si>
+    <t>Mahara Project</t>
+  </si>
+  <si>
+    <t>About ePortfolios</t>
+  </si>
+  <si>
+    <t>Explores how students can collect evidence of learning, reflect on experiences and share work with others.</t>
+  </si>
+  <si>
+    <t>Open-source electronic portfolio platform supporting file uploads, reflections, sharing, comments and feedback.</t>
+  </si>
+  <si>
+    <t>Allows students to collect evidence, explain their learning through reflection, share portfolios with selected users and receive feedback.</t>
+  </si>
+  <si>
+    <t>A portfolio platform is not necessarily configured around daily WIL submission deadlines, mentor approval statuses or coordinator monitoring requirements.</t>
+  </si>
+  <si>
+    <t>Informs TrackWIL's evidence-upload, activity-recording, sharing and feedback features.</t>
+  </si>
+  <si>
+    <t>https://mahara.org/view/view.php?id=3</t>
+  </si>
+  <si>
+    <t>LR04</t>
+  </si>
+  <si>
+    <t>PebblePad</t>
+  </si>
+  <si>
+    <t>PebblePad for assessors</t>
+  </si>
+  <si>
+    <t>Explains how assessors access, review and provide feedback on learner submissions.</t>
+  </si>
+  <si>
+    <t>Online portfolio and assessment platform using ATLAS workspaces, submission lists and assessment tools.</t>
+  </si>
+  <si>
+    <t>Assessors can access learner submissions, provide feedback and use reporting tools to monitor progress and attainment.</t>
+  </si>
+  <si>
+    <t>Access and available actions depend on workspace permissions and institutional configuration. It is primarily an assessment and portfolio workflow rather than a description of TrackWIL's complete WIL process.</t>
+  </si>
+  <si>
+    <t>Informs the design of mentor review screens, feedback functions, submission tracking and staff monitoring dashboards.</t>
+  </si>
+  <si>
+    <t>https://helphub.pebblepad.com/support/solutions/articles/101000539607-pebblepad-for-assessors</t>
+  </si>
+  <si>
+    <t>LR05</t>
+  </si>
+  <si>
+    <t>Mell, P. and Grance, T.</t>
+  </si>
+  <si>
+    <t>The NIST Definition of Cloud Computing</t>
+  </si>
+  <si>
+    <t>Defines cloud computing and describes its characteristics and service and deployment models.</t>
+  </si>
+  <si>
+    <t>Technical definition and classification published as NIST Special Publication 800-145.</t>
+  </si>
+  <si>
+    <t>Cloud computing provides on-demand network access to shared computing resources, which can include servers, storage, applications and networks.</t>
+  </si>
+  <si>
+    <t>Provides a general technical definition rather than a specific hosting recommendation for TrackWIL.</t>
+  </si>
+  <si>
+    <t>Supports the evaluation of cloud hosting for making TrackWIL accessible to students, mentors, coordinators and lecturers.</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.6028/NIST.SP.800-145</t>
+  </si>
+  <si>
+    <t>LR06</t>
+  </si>
+  <si>
+    <t>OWASP Foundation</t>
+  </si>
+  <si>
+    <t>File Upload Cheat Sheet</t>
+  </si>
+  <si>
+    <t>Addresses security risks associated with allowing users to upload files to web applications.</t>
+  </si>
+  <si>
+    <t>Application security guidance covering file validation, allowed extensions, file sizes, storage and access restrictions.</t>
+  </si>
+  <si>
+    <t>Recommends restricting permitted file types, validating uploads, generating safe filenames, limiting file sizes and protecting stored files from unauthorised access.</t>
+  </si>
+  <si>
+    <t>Provides implementation guidance rather than testing results for TrackWIL or a complete security solution.</t>
+  </si>
+  <si>
+    <t>Directly informs the secure implementation of student evidence and document uploads in TrackWIL.</t>
+  </si>
+  <si>
+    <t>https://cheatsheetseries.owasp.org/cheatsheets/File_Upload_Cheat_Sheet.html</t>
+  </si>
+  <si>
+    <t>LR07</t>
+  </si>
+  <si>
+    <t>Authorization Cheat Sheet</t>
+  </si>
+  <si>
+    <t>Addresses the problem of users gaining access to information or actions they are not permitted to use.</t>
+  </si>
+  <si>
+    <t>Application security guidance for implementing and maintaining authorisation controls in software systems.</t>
+  </si>
+  <si>
+    <t>Explains that authentication and authorisation are different. Applications should enforce permissions according to the user's authorised actions and resources.</t>
+  </si>
+  <si>
+    <t>General security guidance; the access rules must still be designed and tested against TrackWIL's specific roles and requirements.</t>
+  </si>
+  <si>
+    <t>Supports role-based access control so students, mentors, coordinators and lecturers can access only the appropriate records and functions.</t>
+  </si>
+  <si>
+    <t>https://cheatsheetseries.owasp.org/cheatsheets/Authorization_Cheat_Sheet.html</t>
+  </si>
+  <si>
+    <t>LR08</t>
+  </si>
+  <si>
+    <t>Authentication Cheat Sheet</t>
+  </si>
+  <si>
+    <t>Addresses secure user authentication and the protection of application accounts.</t>
+  </si>
+  <si>
+    <t>Application security guidance covering authentication practices, credential handling and account protection.</t>
+  </si>
+  <si>
+    <t>Provides recommendations for implementing authentication securely and reducing risks associated with compromised or poorly protected accounts.</t>
+  </si>
+  <si>
+    <t>Does not specify TrackWIL's final authentication technology or provide an evaluation of the completed application.</t>
+  </si>
+  <si>
+    <t>Supports the design of secure registration and login functionality for TrackWIL's different user roles.</t>
+  </si>
+  <si>
+    <t>https://cheatsheetseries.owasp.org/cheatsheets/Authentication_Cheat_Sheet.html</t>
   </si>
 </sst>
 </file>
@@ -443,7 +656,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J38"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -457,7 +670,7 @@
     <col min="10" max="10" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:10" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -471,7 +684,7 @@
       <c r="I1" s="4"/>
       <c r="J1" s="4"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -503,103 +716,263 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="2">
+        <v>2017</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="2">
+        <v>2011</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="C12" s="2"/>
@@ -611,7 +984,7 @@
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -623,7 +996,7 @@
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -635,7 +1008,7 @@
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -647,7 +1020,7 @@
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -659,7 +1032,7 @@
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="2"/>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -671,7 +1044,7 @@
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -683,7 +1056,7 @@
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="2"/>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -695,7 +1068,7 @@
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="2"/>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -707,7 +1080,7 @@
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -719,7 +1092,7 @@
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -731,7 +1104,7 @@
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -743,7 +1116,7 @@
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
       <c r="C24" s="2"/>
@@ -755,7 +1128,7 @@
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="2"/>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -767,7 +1140,7 @@
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="2"/>
       <c r="B26" s="2"/>
       <c r="C26" s="2"/>
@@ -779,7 +1152,7 @@
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="2"/>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
@@ -791,7 +1164,7 @@
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
@@ -803,7 +1176,7 @@
       <c r="I28" s="2"/>
       <c r="J28" s="2"/>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -815,7 +1188,7 @@
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
       <c r="C30" s="2"/>
@@ -827,7 +1200,7 @@
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="C31" s="2"/>
@@ -839,7 +1212,7 @@
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="2"/>
       <c r="B32" s="2"/>
       <c r="C32" s="2"/>
@@ -851,7 +1224,7 @@
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="2"/>
       <c r="B33" s="2"/>
       <c r="C33" s="2"/>
@@ -863,7 +1236,7 @@
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" s="2"/>
       <c r="B34" s="2"/>
       <c r="C34" s="2"/>
@@ -875,7 +1248,7 @@
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="2"/>
       <c r="B35" s="2"/>
       <c r="C35" s="2"/>
@@ -887,7 +1260,7 @@
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
       <c r="C36" s="2"/>
@@ -899,7 +1272,7 @@
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
       <c r="C37" s="2"/>
@@ -911,7 +1284,7 @@
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="2"/>
       <c r="B38" s="2"/>
       <c r="C38" s="2"/>

</xml_diff>